<commit_message>
experience users data update
</commit_message>
<xml_diff>
--- a/Experience/users_data.xlsx
+++ b/Experience/users_data.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20373"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fortineau_Vin\Documents\GitHub\Thesis_report\Experience\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fortineau_vin\Documents\GitHub\Thesis_report\Experience\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A54745-983C-41A7-A569-6F7CDDEE0700}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11775" xr2:uid="{F80D9C69-E636-434F-8593-AF034D74929A}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16200" windowHeight="11700"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>user</t>
   </si>
@@ -39,12 +38,6 @@
     <t>weight</t>
   </si>
   <si>
-    <t>sex</t>
-  </si>
-  <si>
-    <t>right_handed</t>
-  </si>
-  <si>
     <t>racket_sport_practice</t>
   </si>
   <si>
@@ -52,12 +45,6 @@
   </si>
   <si>
     <t>is_first_time</t>
-  </si>
-  <si>
-    <t>m</t>
-  </si>
-  <si>
-    <t>f</t>
   </si>
   <si>
     <t>min</t>
@@ -72,17 +59,26 @@
     <t>mediane</t>
   </si>
   <si>
-    <t>ratio</t>
+    <t>std dev</t>
+  </si>
+  <si>
+    <t>BMI</t>
+  </si>
+  <si>
+    <t>is_male</t>
+  </si>
+  <si>
+    <t>is_right_handed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="000"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -90,16 +86,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -107,13 +117,149 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -427,48 +573,51 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44D288C8-C470-4438-B1FD-DDAF9D8B6C90}">
-  <dimension ref="A1:I61"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="5" max="5" width="7.5703125" customWidth="1"/>
-    <col min="6" max="6" width="14.42578125" customWidth="1"/>
-    <col min="7" max="7" width="22.85546875" customWidth="1"/>
-    <col min="8" max="8" width="22.5703125" customWidth="1"/>
-    <col min="9" max="9" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="7.5703125" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" customWidth="1"/>
+    <col min="8" max="8" width="22.85546875" customWidth="1"/>
+    <col min="9" max="9" width="22.5703125" customWidth="1"/>
+    <col min="10" max="10" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>0</v>
       </c>
       <c r="B2">
@@ -480,23 +629,27 @@
       <c r="D2">
         <v>66</v>
       </c>
-      <c r="E2" t="s">
-        <v>9</v>
+      <c r="E2">
+        <f>D2/(C2/100)^2</f>
+        <v>21.066743273005841</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H2">
         <v>2</v>
       </c>
       <c r="I2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>8</v>
       </c>
@@ -509,8 +662,9 @@
       <c r="D3">
         <v>73</v>
       </c>
-      <c r="E3" t="s">
-        <v>9</v>
+      <c r="E3">
+        <f t="shared" ref="E3:E29" si="0">D3/(C3/100)^2</f>
+        <v>21.798202394816204</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -524,8 +678,11 @@
       <c r="I3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>29</v>
       </c>
@@ -538,23 +695,27 @@
       <c r="D4">
         <v>75</v>
       </c>
-      <c r="E4" t="s">
-        <v>9</v>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>24.212293388429753</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
         <v>2</v>
       </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
       <c r="I4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>50</v>
       </c>
@@ -567,23 +728,27 @@
       <c r="D5">
         <v>70</v>
       </c>
-      <c r="E5" t="s">
-        <v>9</v>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>23.120623596247853</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>113</v>
       </c>
@@ -596,23 +761,27 @@
       <c r="D6">
         <v>70</v>
       </c>
-      <c r="E6" t="s">
-        <v>9</v>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>20.902385858042937</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>160</v>
       </c>
@@ -625,23 +794,27 @@
       <c r="D7">
         <v>85</v>
       </c>
-      <c r="E7" t="s">
-        <v>9</v>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>23.057725694444446</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>194</v>
       </c>
@@ -654,23 +827,27 @@
       <c r="D8">
         <v>59</v>
       </c>
-      <c r="E8" t="s">
-        <v>10</v>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>21.6712580348944</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8">
         <v>0</v>
       </c>
       <c r="I8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>208</v>
       </c>
@@ -683,23 +860,27 @@
       <c r="D9">
         <v>95</v>
       </c>
-      <c r="E9" t="s">
-        <v>9</v>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>29.320987654320987</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>211</v>
       </c>
@@ -712,23 +893,27 @@
       <c r="D10">
         <v>53</v>
       </c>
-      <c r="E10" t="s">
-        <v>10</v>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>19.948059768903612</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
         <v>2</v>
       </c>
-      <c r="H10">
-        <v>1</v>
-      </c>
       <c r="I10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>353</v>
       </c>
@@ -741,23 +926,27 @@
       <c r="D11">
         <v>72</v>
       </c>
-      <c r="E11" t="s">
-        <v>9</v>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>23.243801652892564</v>
       </c>
       <c r="F11">
         <v>1</v>
       </c>
       <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
         <v>2</v>
       </c>
-      <c r="H11">
-        <v>1</v>
-      </c>
       <c r="I11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>364</v>
       </c>
@@ -770,8 +959,9 @@
       <c r="D12">
         <v>68</v>
       </c>
-      <c r="E12" t="s">
-        <v>9</v>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>19.239474875509281</v>
       </c>
       <c r="F12">
         <v>1</v>
@@ -783,10 +973,13 @@
         <v>1</v>
       </c>
       <c r="I12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>378</v>
       </c>
@@ -799,23 +992,27 @@
       <c r="D13">
         <v>75</v>
       </c>
-      <c r="E13" t="s">
-        <v>9</v>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>21.913805697589478</v>
       </c>
       <c r="F13">
         <v>1</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>388</v>
       </c>
@@ -828,24 +1025,28 @@
       <c r="D14">
         <v>90</v>
       </c>
-      <c r="E14" t="s">
-        <v>9</v>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>28.727377190462509</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14">
         <v>0</v>
       </c>
       <c r="H14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
+        <v>1</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
         <v>418</v>
       </c>
       <c r="B15">
@@ -857,24 +1058,28 @@
       <c r="D15">
         <v>60</v>
       </c>
-      <c r="E15" t="s">
-        <v>9</v>
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>19.591836734693878</v>
       </c>
       <c r="F15">
         <v>1</v>
       </c>
       <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
         <v>2</v>
       </c>
-      <c r="H15">
-        <v>0</v>
-      </c>
       <c r="I15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
         <v>456</v>
       </c>
       <c r="B16">
@@ -886,8 +1091,9 @@
       <c r="D16">
         <v>80</v>
       </c>
-      <c r="E16" t="s">
-        <v>9</v>
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>29.031789809841779</v>
       </c>
       <c r="F16">
         <v>1</v>
@@ -901,9 +1107,12 @@
       <c r="I16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
+      <c r="J16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
         <v>495</v>
       </c>
       <c r="B17">
@@ -915,24 +1124,28 @@
       <c r="D17">
         <v>68</v>
       </c>
-      <c r="E17" t="s">
-        <v>9</v>
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>22.460034350640772</v>
       </c>
       <c r="F17">
         <v>1</v>
       </c>
       <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
         <v>2</v>
       </c>
-      <c r="H17">
-        <v>0</v>
-      </c>
       <c r="I17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
         <v>546</v>
       </c>
       <c r="B18">
@@ -944,24 +1157,28 @@
       <c r="D18">
         <v>61</v>
       </c>
-      <c r="E18" t="s">
-        <v>10</v>
+      <c r="E18">
+        <f t="shared" si="0"/>
+        <v>23.243408017070564</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18">
         <v>1</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
         <v>548</v>
       </c>
       <c r="B19">
@@ -973,8 +1190,9 @@
       <c r="D19">
         <v>58</v>
       </c>
-      <c r="E19" t="s">
-        <v>9</v>
+      <c r="E19">
+        <f t="shared" si="0"/>
+        <v>19.157088122605362</v>
       </c>
       <c r="F19">
         <v>1</v>
@@ -986,10 +1204,13 @@
         <v>1</v>
       </c>
       <c r="I19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>555</v>
       </c>
@@ -1002,24 +1223,28 @@
       <c r="D20">
         <v>66</v>
       </c>
-      <c r="E20" t="s">
-        <v>9</v>
+      <c r="E20">
+        <f t="shared" si="0"/>
+        <v>20.598608033457133</v>
       </c>
       <c r="F20">
         <v>1</v>
       </c>
       <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
         <v>2</v>
       </c>
-      <c r="H20">
-        <v>0</v>
-      </c>
       <c r="I20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
         <v>573</v>
       </c>
       <c r="B21">
@@ -1031,24 +1256,28 @@
       <c r="D21">
         <v>70</v>
       </c>
-      <c r="E21" t="s">
-        <v>9</v>
+      <c r="E21">
+        <f t="shared" si="0"/>
+        <v>23.661438615467823</v>
       </c>
       <c r="F21">
         <v>1</v>
       </c>
       <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
         <v>2</v>
       </c>
-      <c r="H21">
-        <v>1</v>
-      </c>
       <c r="I21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
+        <v>1</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
         <v>640</v>
       </c>
       <c r="B22">
@@ -1060,24 +1289,28 @@
       <c r="D22">
         <v>67</v>
       </c>
-      <c r="E22" t="s">
-        <v>10</v>
+      <c r="E22">
+        <f t="shared" si="0"/>
+        <v>20.679012345679013</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
         <v>2</v>
       </c>
-      <c r="H22">
-        <v>0</v>
-      </c>
       <c r="I22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
         <v>661</v>
       </c>
       <c r="B23">
@@ -1089,24 +1322,28 @@
       <c r="D23">
         <v>65</v>
       </c>
-      <c r="E23" t="s">
-        <v>10</v>
+      <c r="E23">
+        <f t="shared" si="0"/>
+        <v>24.767565919829291</v>
       </c>
       <c r="F23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23">
         <v>1</v>
       </c>
       <c r="H23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="2">
         <v>666</v>
       </c>
       <c r="B24">
@@ -1118,8 +1355,9 @@
       <c r="D24">
         <v>95</v>
       </c>
-      <c r="E24" t="s">
-        <v>9</v>
+      <c r="E24">
+        <f t="shared" si="0"/>
+        <v>23.75</v>
       </c>
       <c r="F24">
         <v>1</v>
@@ -1131,10 +1369,13 @@
         <v>1</v>
       </c>
       <c r="I24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>710</v>
       </c>
@@ -1147,8 +1388,9 @@
       <c r="D25">
         <v>105</v>
       </c>
-      <c r="E25" t="s">
-        <v>9</v>
+      <c r="E25">
+        <f t="shared" si="0"/>
+        <v>31.69907016060862</v>
       </c>
       <c r="F25">
         <v>1</v>
@@ -1160,10 +1402,13 @@
         <v>1</v>
       </c>
       <c r="I25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>740</v>
       </c>
@@ -1176,23 +1421,27 @@
       <c r="D26">
         <v>66</v>
       </c>
-      <c r="E26" t="s">
-        <v>9</v>
+      <c r="E26">
+        <f t="shared" si="0"/>
+        <v>22.309356408869661</v>
       </c>
       <c r="F26">
         <v>1</v>
       </c>
       <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
         <v>3</v>
       </c>
-      <c r="H26">
-        <v>0</v>
-      </c>
       <c r="I26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>841</v>
       </c>
@@ -1205,23 +1454,27 @@
       <c r="D27">
         <v>78</v>
       </c>
-      <c r="E27" t="s">
-        <v>9</v>
+      <c r="E27">
+        <f t="shared" si="0"/>
+        <v>23.808797045267237</v>
       </c>
       <c r="F27">
         <v>1</v>
       </c>
       <c r="G27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H27">
         <v>0</v>
       </c>
       <c r="I27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>851</v>
       </c>
@@ -1234,8 +1487,9 @@
       <c r="D28">
         <v>80</v>
       </c>
-      <c r="E28" t="s">
-        <v>9</v>
+      <c r="E28">
+        <f t="shared" si="0"/>
+        <v>23.374726077428779</v>
       </c>
       <c r="F28">
         <v>1</v>
@@ -1244,13 +1498,16 @@
         <v>1</v>
       </c>
       <c r="H28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>922</v>
       </c>
@@ -1263,8 +1520,9 @@
       <c r="D29">
         <v>60</v>
       </c>
-      <c r="E29" t="s">
-        <v>9</v>
+      <c r="E29">
+        <f t="shared" si="0"/>
+        <v>20.761245674740486</v>
       </c>
       <c r="F29">
         <v>1</v>
@@ -1273,181 +1531,260 @@
         <v>1</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B31">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B31" s="6">
         <f>MIN(B2:B29)</f>
         <v>19</v>
       </c>
-      <c r="C31">
+      <c r="C31" s="6">
         <f>MIN(C2:C29)</f>
         <v>162</v>
       </c>
-      <c r="D31">
+      <c r="D31" s="6">
         <f>MIN(D2:D29)</f>
         <v>53</v>
       </c>
-      <c r="G31">
-        <f>MIN(G2:G29)</f>
-        <v>0</v>
-      </c>
-      <c r="H31">
+      <c r="E31" s="6">
+        <f>MIN(E2:E29)</f>
+        <v>19.157088122605362</v>
+      </c>
+      <c r="F31" s="6">
+        <f t="shared" ref="F31:G31" si="1">MIN(F2:F29)</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="6">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H31" s="6">
         <f>MIN(H2:H29)</f>
         <v>0</v>
       </c>
-      <c r="I31">
+      <c r="I31" s="6">
         <f>MIN(I2:I29)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B32">
+      <c r="J31" s="7">
+        <f>MIN(J2:J29)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B32" s="8">
         <f>MAX(B2:B29)</f>
         <v>56</v>
       </c>
-      <c r="C32">
+      <c r="C32" s="8">
         <f>MAX(C2:C29)</f>
         <v>200</v>
       </c>
-      <c r="D32">
+      <c r="D32" s="8">
         <f>MAX(D2:D29)</f>
         <v>105</v>
       </c>
-      <c r="G32">
-        <f>MAX(G2:G29)</f>
+      <c r="E32" s="8">
+        <f>MAX(E2:E29)</f>
+        <v>31.69907016060862</v>
+      </c>
+      <c r="F32" s="8">
+        <f t="shared" ref="F32:G32" si="2">MAX(F2:F29)</f>
+        <v>1</v>
+      </c>
+      <c r="G32" s="8">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="H32" s="8">
+        <f>MAX(H2:H29)</f>
         <v>3</v>
       </c>
-      <c r="H32">
-        <f>MAX(H2:H29)</f>
+      <c r="I32" s="8">
+        <f>MAX(I2:I29)</f>
         <v>2</v>
       </c>
-      <c r="I32">
-        <f>MAX(I2:I29)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B33">
+      <c r="J32" s="9">
+        <f>MAX(J2:J29)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B33" s="8">
         <f>AVERAGE(B2:B29)</f>
         <v>30.214285714285715</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="8">
         <f>AVERAGE(C2:C29)</f>
         <v>176.89285714285714</v>
       </c>
-      <c r="D33">
+      <c r="D33" s="8">
         <f>AVERAGE(D2:D29)</f>
         <v>72.5</v>
       </c>
-      <c r="G33">
+      <c r="E33" s="8">
+        <f>AVERAGE(E2:E29)</f>
+        <v>23.111311299848584</v>
+      </c>
+      <c r="F33" s="8">
+        <f>AVERAGE(F2:F29)</f>
+        <v>0.8214285714285714</v>
+      </c>
+      <c r="G33" s="8">
         <f>AVERAGE(G2:G29)</f>
+        <v>0.8928571428571429</v>
+      </c>
+      <c r="H33" s="8">
+        <f>AVERAGE(H2:H29)</f>
         <v>1.1428571428571428</v>
       </c>
-      <c r="H33">
-        <f>AVERAGE(H2:H29)</f>
+      <c r="I33" s="8">
+        <f>AVERAGE(I2:I29)</f>
         <v>0.5714285714285714</v>
       </c>
-      <c r="I33">
-        <f>AVERAGE(I2:I29)</f>
+      <c r="J33" s="9">
+        <f>AVERAGE(J2:J29)</f>
         <v>0.6071428571428571</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B34">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34" s="8">
         <f>MEDIAN(B2:B29)</f>
         <v>27</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="8">
         <f>MEDIAN(C2:C29)</f>
         <v>176.5</v>
       </c>
-      <c r="D34">
+      <c r="D34" s="8">
         <f>MEDIAN(D2:D29)</f>
         <v>70</v>
       </c>
-      <c r="G34">
+      <c r="E34" s="8">
+        <f>MEDIAN(E2:E29)</f>
+        <v>22.758880022542609</v>
+      </c>
+      <c r="F34" s="8">
+        <f>MEDIAN(F2:F29)</f>
+        <v>1</v>
+      </c>
+      <c r="G34" s="8">
         <f>MEDIAN(G2:G29)</f>
         <v>1</v>
       </c>
-      <c r="H34">
+      <c r="H34" s="8">
         <f>MEDIAN(H2:H29)</f>
         <v>1</v>
       </c>
-      <c r="I34">
+      <c r="I34" s="8">
         <f>MEDIAN(I2:I29)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E35">
-        <f>COUNTIF(E2:E29,"f")/COUNTA(E2:E29)</f>
-        <v>0.17857142857142858</v>
-      </c>
-      <c r="F35">
-        <f>COUNTIF(F2:F29,0)/COUNTA(E2:E29)</f>
-        <v>0.10714285714285714</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J34" s="9">
+        <f>MEDIAN(J2:J29)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B35" s="10">
+        <f>_xlfn.STDEV.S(B3:B30)</f>
+        <v>9.0596315088927923</v>
+      </c>
+      <c r="C35" s="10">
+        <f>_xlfn.STDEV.S(C3:C30)</f>
+        <v>9.1581545560115387</v>
+      </c>
+      <c r="D35" s="10">
+        <f>_xlfn.STDEV.S(D3:D30)</f>
+        <v>12.608277478254569</v>
+      </c>
+      <c r="E35" s="10">
+        <f>_xlfn.STDEV.S(E3:E30)</f>
+        <v>3.1983045780777366</v>
+      </c>
+      <c r="F35" s="10">
+        <f>_xlfn.STDEV.S(F3:F30)</f>
+        <v>0.3958473906635695</v>
+      </c>
+      <c r="G35" s="10">
+        <f>_xlfn.STDEV.S(G3:G30)</f>
+        <v>0.26688025634181184</v>
+      </c>
+      <c r="H35" s="10">
+        <f>_xlfn.STDEV.S(H3:H30)</f>
+        <v>0.84731854573632337</v>
+      </c>
+      <c r="I35" s="10">
+        <f>_xlfn.STDEV.S(I3:I30)</f>
+        <v>0.50917507721731559</v>
+      </c>
+      <c r="J35" s="11">
+        <f>_xlfn.STDEV.S(J3:J30)</f>
+        <v>0.49210287762341132</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
@@ -1489,7 +1826,11 @@
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" s="1"/>
     </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="1"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
experimental user data update
</commit_message>
<xml_diff>
--- a/Experience/users_data.xlsx
+++ b/Experience/users_data.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20373"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fortineau_Vin\Documents\GitHub\Thesis_report\Experience\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fortineau_vin\Documents\GitHub\Thesis_report\Experience\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C93159FA-9122-4AAA-9A6F-0ACED37EC499}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16200" windowHeight="11700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16200" windowHeight="11700"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>user</t>
   </si>
@@ -71,11 +70,17 @@
   <si>
     <t>is_right_handed</t>
   </si>
+  <si>
+    <t>date exp 1</t>
+  </si>
+  <si>
+    <t>date exp 2</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="000"/>
   </numFmts>
@@ -96,7 +101,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -106,6 +111,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -245,7 +262,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -261,6 +278,10 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -574,8 +595,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J65"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="7.5703125" customWidth="1"/>
@@ -585,7 +606,7 @@
     <col min="10" max="10" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -616,23 +637,29 @@
       <c r="J1" s="5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+      <c r="K1" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="L1" s="15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="18">
         <v>0</v>
       </c>
       <c r="B2">
         <v>27</v>
       </c>
       <c r="C2">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D2">
         <v>66</v>
       </c>
       <c r="E2">
         <f>D2/(C2/100)^2</f>
-        <v>21.066743273005841</v>
+        <v>21.551020408163264</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -649,8 +676,14 @@
       <c r="J2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K2" s="16">
+        <v>44357</v>
+      </c>
+      <c r="L2" s="16">
+        <v>44357</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>8</v>
       </c>
@@ -682,8 +715,14 @@
       <c r="J3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K3" s="16">
+        <v>44355</v>
+      </c>
+      <c r="L3" s="16">
+        <v>44355</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>29</v>
       </c>
@@ -715,9 +754,15 @@
       <c r="J4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+      <c r="K4" s="16">
+        <v>44341</v>
+      </c>
+      <c r="L4" s="16">
+        <v>44341</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="17">
         <v>41</v>
       </c>
       <c r="B5">
@@ -748,8 +793,14 @@
       <c r="J5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K5" s="16">
+        <v>44363</v>
+      </c>
+      <c r="L5" s="16">
+        <v>44363</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>50</v>
       </c>
@@ -781,8 +832,14 @@
       <c r="J6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K6" s="16">
+        <v>44350</v>
+      </c>
+      <c r="L6" s="16">
+        <v>44350</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>113</v>
       </c>
@@ -814,8 +871,14 @@
       <c r="J7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K7" s="16">
+        <v>44354</v>
+      </c>
+      <c r="L7" s="16">
+        <v>44354</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>160</v>
       </c>
@@ -847,8 +910,14 @@
       <c r="J8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K8" s="16">
+        <v>44350</v>
+      </c>
+      <c r="L8" s="16">
+        <v>44350</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>194</v>
       </c>
@@ -880,8 +949,14 @@
       <c r="J9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K9" s="16">
+        <v>44348</v>
+      </c>
+      <c r="L9" s="16">
+        <v>44350</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>208</v>
       </c>
@@ -913,9 +988,15 @@
       <c r="J10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
+      <c r="K10" s="16">
+        <v>44354</v>
+      </c>
+      <c r="L10" s="16">
+        <v>44354</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="17">
         <v>211</v>
       </c>
       <c r="B11">
@@ -946,9 +1027,15 @@
       <c r="J11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
+      <c r="K11" s="16">
+        <v>44349</v>
+      </c>
+      <c r="L11" s="16">
+        <v>44349</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="17">
         <v>278</v>
       </c>
       <c r="B12">
@@ -979,8 +1066,14 @@
       <c r="J12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K12" s="16">
+        <v>44349</v>
+      </c>
+      <c r="L12" s="16">
+        <v>44349</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>311</v>
       </c>
@@ -1012,8 +1105,14 @@
       <c r="J13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K13" s="16">
+        <v>44371</v>
+      </c>
+      <c r="L13" s="16">
+        <v>44371</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>353</v>
       </c>
@@ -1045,8 +1144,14 @@
       <c r="J14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K14" s="16">
+        <v>44349</v>
+      </c>
+      <c r="L14" s="16">
+        <v>44349</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>364</v>
       </c>
@@ -1078,8 +1183,14 @@
       <c r="J15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K15" s="16">
+        <v>44354</v>
+      </c>
+      <c r="L15" s="16">
+        <v>44354</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>378</v>
       </c>
@@ -1111,8 +1222,14 @@
       <c r="J16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K16" s="16">
+        <v>44343</v>
+      </c>
+      <c r="L16" s="16">
+        <v>44343</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>388</v>
       </c>
@@ -1144,8 +1261,14 @@
       <c r="J17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K17" s="16">
+        <v>44343</v>
+      </c>
+      <c r="L17" s="16">
+        <v>44343</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>418</v>
       </c>
@@ -1177,8 +1300,14 @@
       <c r="J18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K18" s="16">
+        <v>44348</v>
+      </c>
+      <c r="L18" s="16">
+        <v>44348</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>456</v>
       </c>
@@ -1210,8 +1339,14 @@
       <c r="J19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K19" s="16">
+        <v>44348</v>
+      </c>
+      <c r="L19" s="16">
+        <v>44348</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>495</v>
       </c>
@@ -1243,8 +1378,14 @@
       <c r="J20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K20" s="16">
+        <v>44351</v>
+      </c>
+      <c r="L20" s="16">
+        <v>44351</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>546</v>
       </c>
@@ -1276,8 +1417,14 @@
       <c r="J21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K21" s="16">
+        <v>44351</v>
+      </c>
+      <c r="L21" s="16">
+        <v>44348</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>548</v>
       </c>
@@ -1309,9 +1456,15 @@
       <c r="J22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
+      <c r="K22" s="16">
+        <v>44349</v>
+      </c>
+      <c r="L22" s="16">
+        <v>44349</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" s="17">
         <v>555</v>
       </c>
       <c r="B23">
@@ -1342,8 +1495,14 @@
       <c r="J23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K23" s="16">
+        <v>44356</v>
+      </c>
+      <c r="L23" s="16">
+        <v>44356</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>573</v>
       </c>
@@ -1375,8 +1534,14 @@
       <c r="J24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K24" s="16">
+        <v>44349</v>
+      </c>
+      <c r="L24" s="16">
+        <v>44349</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>640</v>
       </c>
@@ -1408,8 +1573,14 @@
       <c r="J25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K25" s="16">
+        <v>44351</v>
+      </c>
+      <c r="L25" s="16">
+        <v>44351</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>661</v>
       </c>
@@ -1441,8 +1612,14 @@
       <c r="J26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K26" s="16">
+        <v>44348</v>
+      </c>
+      <c r="L26" s="16">
+        <v>44348</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>666</v>
       </c>
@@ -1474,8 +1651,14 @@
       <c r="J27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K27" s="16">
+        <v>44349</v>
+      </c>
+      <c r="L27" s="16">
+        <v>44349</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>710</v>
       </c>
@@ -1507,8 +1690,14 @@
       <c r="J28">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K28" s="16">
+        <v>44355</v>
+      </c>
+      <c r="L28" s="16">
+        <v>44355</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>740</v>
       </c>
@@ -1540,8 +1729,14 @@
       <c r="J29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K29" s="16">
+        <v>44350</v>
+      </c>
+      <c r="L29" s="16">
+        <v>44350</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>841</v>
       </c>
@@ -1573,8 +1768,14 @@
       <c r="J30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K30" s="16">
+        <v>44351</v>
+      </c>
+      <c r="L30" s="16">
+        <v>44351</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>851</v>
       </c>
@@ -1606,8 +1807,14 @@
       <c r="J31">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K31" s="16">
+        <v>44351</v>
+      </c>
+      <c r="L31" s="16">
+        <v>44351</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>922</v>
       </c>
@@ -1638,6 +1845,12 @@
       </c>
       <c r="J32">
         <v>0</v>
+      </c>
+      <c r="K32" s="16">
+        <v>44355</v>
+      </c>
+      <c r="L32" s="16">
+        <v>44350</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1735,7 +1948,7 @@
       </c>
       <c r="C36" s="8">
         <f t="shared" si="3"/>
-        <v>176.2258064516129</v>
+        <v>176.16129032258064</v>
       </c>
       <c r="D36" s="8">
         <f t="shared" si="3"/>
@@ -1743,7 +1956,7 @@
       </c>
       <c r="E36" s="8">
         <f t="shared" si="3"/>
-        <v>22.869707507414624</v>
+        <v>22.885329350484216</v>
       </c>
       <c r="F36" s="8">
         <f t="shared" si="3"/>

</xml_diff>